<commit_message>
feat(instruments)!: build products explicitly
Add MakeInstrument readiness and date resolution, with shared build_using
orchestration. Resolve dates and initial loan observations before pricing
across Rust, Python and Excel. Keep prepayment models generic over scalars.

BREAKING CHANGE: replace Resolve, ResolutionContext and deferred trades
with maker.build() or maker.build_using(context). Import MakeInstrument
for Rust maker methods. Excel constructors require a pricing context.
</commit_message>
<xml_diff>
--- a/bindings/excel/examples/workbooks/bond_pricing_example.xlsx
+++ b/bindings/excel/examples/workbooks/bond_pricing_example.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d6018bc907cdb526/Escritorio/Pega/quantsupport/bindings/excel/examples/workbooks/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_315D2BFE280CEF1796A1F0088F2236289BE1A375" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{240D7125-1DB9-499E-A07C-517DADC7E1FB}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Start Here" sheetId="1" r:id="rId1"/>
@@ -22,7 +16,6 @@
     <sheet name="6 Risk" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Start Here'!$A$1:$F$29</definedName>
     <definedName name="Bond_BaseCurves">'2 Market'!$B$21</definedName>
     <definedName name="Bond_C01_Anchor">'1 Inputs'!$B$17</definedName>
     <definedName name="Bond_C01_AnchorValue">'1 Inputs'!$C$17</definedName>
@@ -67,6 +60,7 @@
     <definedName name="Bond_Start">'1 Inputs'!$B$8</definedName>
     <definedName name="Bond_ValuationDate">'1 Inputs'!$B$7</definedName>
     <definedName name="Bond_ZeroRates">'2 Market'!$B$7:$B$11</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Start Here'!$A$1:$F$29</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'1 Inputs'!$1:$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'2 Market'!$1:$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'3 Build'!$1:$6</definedName>
@@ -74,30 +68,17 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'5 Cashflows'!$1:$7</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'6 Risk'!$1:$7</definedName>
   </definedNames>
-  <calcPr calcId="191029" forceFullCalc="1"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author/>
   </authors>
   <commentList>
-    <comment ref="B7" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
+    <comment ref="B7" authorId="0">
       <text>
         <r>
           <rPr>
@@ -110,7 +91,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B8" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000002000000}">
+    <comment ref="B8" authorId="0">
       <text>
         <r>
           <rPr>
@@ -123,7 +104,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B9" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000003000000}">
+    <comment ref="B9" authorId="0">
       <text>
         <r>
           <rPr>
@@ -136,7 +117,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B10" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000004000000}">
+    <comment ref="B10" authorId="0">
       <text>
         <r>
           <rPr>
@@ -149,7 +130,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B11" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000005000000}">
+    <comment ref="B11" authorId="0">
       <text>
         <r>
           <rPr>
@@ -162,7 +143,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B12" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000006000000}">
+    <comment ref="B12" authorId="0">
       <text>
         <r>
           <rPr>
@@ -180,12 +161,12 @@
 </file>
 
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author/>
   </authors>
   <commentList>
-    <comment ref="B18" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000001000000}">
+    <comment ref="B18" authorId="0">
       <text>
         <r>
           <rPr>
@@ -198,7 +179,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B21" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000002000000}">
+    <comment ref="B21" authorId="0">
       <text>
         <r>
           <rPr>
@@ -216,12 +197,12 @@
 </file>
 
 <file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author/>
   </authors>
   <commentList>
-    <comment ref="B7" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000001000000}">
+    <comment ref="B7" authorId="0">
       <text>
         <r>
           <rPr>
@@ -234,7 +215,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B10" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000002000000}">
+    <comment ref="B10" authorId="0">
       <text>
         <r>
           <rPr>
@@ -247,7 +228,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B13" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000003000000}">
+    <comment ref="B13" authorId="0">
       <text>
         <r>
           <rPr>
@@ -260,7 +241,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B16" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000004000000}">
+    <comment ref="B16" authorId="0">
       <text>
         <r>
           <rPr>
@@ -273,7 +254,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B19" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000005000000}">
+    <comment ref="B19" authorId="0">
       <text>
         <r>
           <rPr>
@@ -286,7 +267,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B22" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000006000000}">
+    <comment ref="B22" authorId="0">
       <text>
         <r>
           <rPr>
@@ -299,7 +280,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B25" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000007000000}">
+    <comment ref="B25" authorId="0">
       <text>
         <r>
           <rPr>
@@ -312,7 +293,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B28" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000008000000}">
+    <comment ref="B28" authorId="0">
       <text>
         <r>
           <rPr>
@@ -325,7 +306,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B31" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000009000000}">
+    <comment ref="B31" authorId="0">
       <text>
         <r>
           <rPr>
@@ -338,7 +319,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B34" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-00000A000000}">
+    <comment ref="B34" authorId="0">
       <text>
         <r>
           <rPr>
@@ -351,7 +332,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B45" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-00000B000000}">
+    <comment ref="B45" authorId="0">
       <text>
         <r>
           <rPr>
@@ -822,13 +803,15 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="#,##0.00;[Red]\(#,##0.00\)"/>
-    <numFmt numFmtId="165" formatCode="0.0000"/>
-    <numFmt numFmtId="166" formatCode="0.0000%"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="5">
+    <numFmt numFmtId="164" formatCode="#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="0.00%"/>
+    <numFmt numFmtId="166" formatCode="#,##0.00;[Red](#,##0.00)"/>
+    <numFmt numFmtId="167" formatCode="0.0000"/>
+    <numFmt numFmtId="168" formatCode="0.0000%"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1002,9 +985,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1028,52 +1017,22 @@
     <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="8" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="8" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="8" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="9" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="9" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="9" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1082,21 +1041,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1134,7 +1085,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -1168,7 +1119,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -1203,10 +1153,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1379,12 +1328,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F29"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="26.1" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="26.25" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="8.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="22.7109375" style="1" customWidth="1"/>
@@ -1393,257 +1342,257 @@
     <col min="6" max="6" width="18.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+    <row r="1" spans="1:6" ht="30" customHeight="1">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-    </row>
-    <row r="2" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15"/>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-    </row>
-    <row r="3" spans="1:6" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="16" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+    </row>
+    <row r="2" spans="1:6" ht="30" customHeight="1">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+    </row>
+    <row r="3" spans="1:6" ht="26.25" customHeight="1">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-    </row>
-    <row r="4" spans="1:6" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="16"/>
-      <c r="B4" s="16"/>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="16"/>
-    </row>
-    <row r="6" spans="1:6" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="24" t="s">
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+    </row>
+    <row r="4" spans="1:6" ht="26.25" customHeight="1">
+      <c r="A4" s="3"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+    </row>
+    <row r="6" spans="1:6" ht="26.25" customHeight="1">
+      <c r="A6" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="24"/>
-      <c r="C6" s="24"/>
-      <c r="D6" s="24"/>
-      <c r="E6" s="24"/>
-      <c r="F6" s="24"/>
-    </row>
-    <row r="7" spans="1:6" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="24"/>
-      <c r="B7" s="24"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24"/>
-    </row>
-    <row r="9" spans="1:6" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="17" t="s">
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+    </row>
+    <row r="7" spans="1:6" ht="26.25" customHeight="1">
+      <c r="A7" s="4"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+    </row>
+    <row r="9" spans="1:6" ht="26.25" customHeight="1">
+      <c r="A9" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="17"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-    </row>
-    <row r="10" spans="1:6" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+    </row>
+    <row r="10" spans="1:6" ht="33.75" customHeight="1">
+      <c r="A10" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C10" s="19"/>
-      <c r="D10" s="18" t="s">
+      <c r="C10" s="7"/>
+      <c r="D10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
-    </row>
-    <row r="11" spans="1:6" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+    </row>
+    <row r="11" spans="1:6" ht="33.75" customHeight="1">
+      <c r="A11" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="23" t="s">
+      <c r="B11" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C11" s="19"/>
-      <c r="D11" s="18" t="s">
+      <c r="C11" s="7"/>
+      <c r="D11" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E11" s="18"/>
-      <c r="F11" s="18"/>
-    </row>
-    <row r="12" spans="1:6" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+    </row>
+    <row r="12" spans="1:6" ht="33.75" customHeight="1">
+      <c r="A12" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="23" t="s">
+      <c r="B12" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="18" t="s">
+      <c r="C12" s="7"/>
+      <c r="D12" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
-    </row>
-    <row r="13" spans="1:6" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+    </row>
+    <row r="13" spans="1:6" ht="33.75" customHeight="1">
+      <c r="A13" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="23" t="s">
+      <c r="B13" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="19"/>
-      <c r="D13" s="18" t="s">
+      <c r="C13" s="7"/>
+      <c r="D13" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
-    </row>
-    <row r="14" spans="1:6" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+    </row>
+    <row r="14" spans="1:6" ht="33.75" customHeight="1">
+      <c r="A14" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="23" t="s">
+      <c r="B14" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="18" t="s">
+      <c r="C14" s="7"/>
+      <c r="D14" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
-    </row>
-    <row r="15" spans="1:6" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+    </row>
+    <row r="15" spans="1:6" ht="33.75" customHeight="1">
+      <c r="A15" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B15" s="23" t="s">
+      <c r="B15" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="19"/>
-      <c r="D15" s="18" t="s">
+      <c r="C15" s="7"/>
+      <c r="D15" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E15" s="18"/>
-      <c r="F15" s="18"/>
-    </row>
-    <row r="18" spans="1:6" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="17" t="s">
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+    </row>
+    <row r="18" spans="1:6" ht="26.25" customHeight="1">
+      <c r="A18" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="17"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
-    </row>
-    <row r="19" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="20" t="s">
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+    </row>
+    <row r="19" spans="1:6" ht="30" customHeight="1">
+      <c r="A19" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="B19" s="20"/>
-      <c r="C19" s="20"/>
-      <c r="D19" s="18" t="s">
+      <c r="B19" s="8"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E19" s="18"/>
-      <c r="F19" s="18"/>
-    </row>
-    <row r="20" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="21" t="s">
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+    </row>
+    <row r="20" spans="1:6" ht="30" customHeight="1">
+      <c r="A20" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="B20" s="21"/>
-      <c r="C20" s="21"/>
-      <c r="D20" s="18" t="s">
+      <c r="B20" s="9"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E20" s="18"/>
-      <c r="F20" s="18"/>
-    </row>
-    <row r="21" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="22" t="s">
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+    </row>
+    <row r="21" spans="1:6" ht="30" customHeight="1">
+      <c r="A21" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B21" s="22"/>
-      <c r="C21" s="22"/>
-      <c r="D21" s="18" t="s">
+      <c r="B21" s="10"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="E21" s="18"/>
-      <c r="F21" s="18"/>
-    </row>
-    <row r="23" spans="1:6" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="17" t="s">
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+    </row>
+    <row r="23" spans="1:6" ht="26.25" customHeight="1">
+      <c r="A23" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B23" s="17"/>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
-      <c r="F23" s="17"/>
-    </row>
-    <row r="24" spans="1:6" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="18" t="s">
+      <c r="B23" s="5"/>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+    </row>
+    <row r="24" spans="1:6" ht="33.75" customHeight="1">
+      <c r="A24" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="18"/>
-      <c r="C24" s="18"/>
-      <c r="D24" s="18"/>
-      <c r="E24" s="18"/>
-      <c r="F24" s="18"/>
-    </row>
-    <row r="25" spans="1:6" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="18" t="s">
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+      <c r="F24" s="1"/>
+    </row>
+    <row r="25" spans="1:6" ht="33.75" customHeight="1">
+      <c r="A25" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B25" s="18"/>
-      <c r="C25" s="18"/>
-      <c r="D25" s="18"/>
-      <c r="E25" s="18"/>
-      <c r="F25" s="18"/>
-    </row>
-    <row r="26" spans="1:6" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="18" t="s">
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+      <c r="F25" s="1"/>
+    </row>
+    <row r="26" spans="1:6" ht="33.75" customHeight="1">
+      <c r="A26" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B26" s="18"/>
-      <c r="C26" s="18"/>
-      <c r="D26" s="18"/>
-      <c r="E26" s="18"/>
-      <c r="F26" s="18"/>
-    </row>
-    <row r="28" spans="1:6" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="19" t="s">
+      <c r="B26" s="1"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+    </row>
+    <row r="28" spans="1:6" ht="26.25" customHeight="1">
+      <c r="A28" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="19"/>
-      <c r="C28" s="19"/>
-      <c r="D28" s="19"/>
-      <c r="E28" s="19"/>
-      <c r="F28" s="19"/>
-    </row>
-    <row r="29" spans="1:6" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="19"/>
-      <c r="B29" s="19"/>
-      <c r="C29" s="19"/>
-      <c r="D29" s="19"/>
-      <c r="E29" s="19"/>
-      <c r="F29" s="19"/>
+      <c r="B28" s="7"/>
+      <c r="C28" s="7"/>
+      <c r="D28" s="7"/>
+      <c r="E28" s="7"/>
+      <c r="F28" s="7"/>
+    </row>
+    <row r="29" spans="1:6" ht="26.25" customHeight="1">
+      <c r="A29" s="7"/>
+      <c r="B29" s="7"/>
+      <c r="C29" s="7"/>
+      <c r="D29" s="7"/>
+      <c r="E29" s="7"/>
+      <c r="F29" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="28">
@@ -1677,12 +1626,12 @@
     <mergeCell ref="A28:F29"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B10" location="'1 Inputs'!A1" display="1 Inputs" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="B11" location="'2 Market'!A1" display="2 Market" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="B12" location="'3 Build'!A1" display="3 Build" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="B13" location="'4 Results'!A1" display="4 Results" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="B14" location="'5 Cashflows'!A1" display="5 Cashflows" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="B15" location="'6 Risk'!A1" display="6 Risk" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="B10" location="'1 Inputs'!A1" display="1 Inputs"/>
+    <hyperlink ref="B11" location="'2 Market'!A1" display="2 Market"/>
+    <hyperlink ref="B12" location="'3 Build'!A1" display="3 Build"/>
+    <hyperlink ref="B13" location="'4 Results'!A1" display="4 Results"/>
+    <hyperlink ref="B14" location="'5 Cashflows'!A1" display="5 Cashflows"/>
+    <hyperlink ref="B15" location="'6 Risk'!A1" display="6 Risk"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
@@ -1690,230 +1639,230 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <tabColor rgb="FF337AB7"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:C31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="24" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="24" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="34.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="26.7109375" style="1" customWidth="1"/>
     <col min="3" max="3" width="62.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+    <row r="1" spans="1:3" ht="38.25" customHeight="1">
+      <c r="A1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-    </row>
-    <row r="2" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+    </row>
+    <row r="2" spans="1:3" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-    </row>
-    <row r="3" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="16"/>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-    </row>
-    <row r="4" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+    </row>
+    <row r="3" spans="1:3" ht="24" customHeight="1">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+    </row>
+    <row r="4" spans="1:3" ht="36" customHeight="1">
+      <c r="A4" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+    <row r="6" spans="1:3" ht="36" customHeight="1">
+      <c r="A6" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="5" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="32.25" customHeight="1">
       <c r="A7" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="7" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="32.25" customHeight="1">
       <c r="A8" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="7" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="32.25" customHeight="1">
       <c r="A9" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="7" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" ht="32.25" customHeight="1">
       <c r="A10" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B10" s="9">
+      <c r="B10" s="11">
         <v>1000000</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="7" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="32.25" customHeight="1">
       <c r="A11" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B11" s="10">
+      <c r="B11" s="12">
         <v>0.04</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="7" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="32.25" customHeight="1">
       <c r="A12" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="7" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
+    <row r="16" spans="1:3" ht="36" customHeight="1">
+      <c r="A16" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" ht="24" customHeight="1">
       <c r="A17" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="C17" s="10">
+      <c r="C17" s="12">
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" ht="24" customHeight="1">
       <c r="A18" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="C18" s="10">
+      <c r="C18" s="12">
         <v>0.01</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" ht="24" customHeight="1">
       <c r="A19" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="C19" s="9">
+      <c r="C19" s="11">
         <v>100</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
+    <row r="22" spans="1:3" ht="36" customHeight="1">
+      <c r="A22" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="C22" s="3"/>
-    </row>
-    <row r="23" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C22" s="5"/>
+    </row>
+    <row r="23" spans="1:3" ht="24" customHeight="1">
       <c r="A23" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="7" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" ht="24" customHeight="1">
       <c r="A24" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="7" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" ht="24" customHeight="1">
       <c r="A25" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="7" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" ht="24" customHeight="1">
       <c r="A26" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="7" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" ht="24" customHeight="1">
       <c r="A27" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="7" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="3" t="s">
+    <row r="30" spans="1:3" ht="36" customHeight="1">
+      <c r="A30" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="B30" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="C30" s="3"/>
-    </row>
-    <row r="31" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C30" s="5"/>
+    </row>
+    <row r="31" spans="1:3" ht="24" customHeight="1">
       <c r="A31" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B31" s="8" t="s">
         <v>77</v>
       </c>
     </row>
@@ -1923,8 +1872,8 @@
     <mergeCell ref="A2:C3"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A4" location="'Start Here'!A1" display="← Start Here" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
-    <hyperlink ref="C4" location="'2 Market'!A1" display="Next → 2 Market" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
+    <hyperlink ref="A4" location="'Start Here'!A1" display="← Start Here"/>
+    <hyperlink ref="C4" location="'2 Market'!A1" display="Next → 2 Market"/>
   </hyperlinks>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape"/>
@@ -1936,157 +1885,157 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <tabColor rgb="FF337AB7"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:C22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="24" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="24" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="38.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="42.7109375" style="1" customWidth="1"/>
     <col min="3" max="3" width="44.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+    <row r="1" spans="1:3" ht="38.25" customHeight="1">
+      <c r="A1" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-    </row>
-    <row r="2" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+    </row>
+    <row r="2" spans="1:3" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-    </row>
-    <row r="3" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="16"/>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-    </row>
-    <row r="4" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+    </row>
+    <row r="3" spans="1:3" ht="24" customHeight="1">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+    </row>
+    <row r="4" spans="1:3" ht="36" customHeight="1">
+      <c r="A4" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="6" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+    <row r="6" spans="1:3" ht="36" customHeight="1">
+      <c r="A6" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="C6" s="3"/>
-    </row>
-    <row r="7" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+      <c r="C6" s="5"/>
+    </row>
+    <row r="7" spans="1:3" ht="24" customHeight="1">
+      <c r="A7" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="12">
         <v>0.03</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
+    <row r="8" spans="1:3" ht="24" customHeight="1">
+      <c r="A8" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="B8" s="10">
+      <c r="B8" s="12">
         <v>0.03</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
+    <row r="9" spans="1:3" ht="24" customHeight="1">
+      <c r="A9" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="B9" s="10">
-        <v>3.2000000000000001E-2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
+      <c r="B9" s="12">
+        <v>0.032</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="24" customHeight="1">
+      <c r="A10" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="B10" s="10">
-        <v>3.4000000000000002E-2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
+      <c r="B10" s="12">
+        <v>0.034</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="24" customHeight="1">
+      <c r="A11" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="B11" s="10">
-        <v>3.5000000000000003E-2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="19" t="s">
+      <c r="B11" s="12">
+        <v>0.035</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="24" customHeight="1">
+      <c r="A13" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="B13" s="19"/>
-      <c r="C13" s="19"/>
-    </row>
-    <row r="14" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="19"/>
-      <c r="B14" s="19"/>
-      <c r="C14" s="19"/>
-    </row>
-    <row r="17" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
+    </row>
+    <row r="14" spans="1:3" ht="24" customHeight="1">
+      <c r="A14" s="7"/>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+    </row>
+    <row r="17" spans="1:3" ht="36" customHeight="1">
+      <c r="A17" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="5" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
+    <row r="18" spans="1:3" ht="38.25" customHeight="1">
+      <c r="A18" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="B18" s="8" t="e" cm="1">
-        <f t="array" aca="1" ref="B18" ca="1">_xll.QS.CONTEXT.CREATE("Bond.Root",Bond_ValuationDate,"USD","SOFR")</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C18" s="5" t="s">
+      <c r="B18" s="10" cm="1" t="str">
+        <f t="array" ref="B18">_xll.QS.CONTEXT.CREATE("Bond.Root",Bond_ValuationDate,"USD","SOFR")</f>
+        <v/>
+      </c>
+      <c r="C18" s="7" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="14" t="str">
-        <f ca="1">SUBSTITUTE(_xlfn.FORMULATEXT(B18),",",", ")</f>
-        <v>=QS.CONTEXT.CREATE("Bond.Root";Bond_ValuationDate;"USD";"SOFR")</v>
-      </c>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-    </row>
-    <row r="21" spans="1:3" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="2" t="s">
+    <row r="19" spans="1:3" ht="33.75" customHeight="1">
+      <c r="A19" s="13" t="str">
+        <f>SUBSTITUTE(_xlfn.FORMULATEXT(B18),",",", ")</f>
+        <v>=QS.CONTEXT.CREATE("Bond.Root", Bond_ValuationDate, "USD", "SOFR")</v>
+      </c>
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+    </row>
+    <row r="21" spans="1:3" ht="38.25" customHeight="1">
+      <c r="A21" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="B21" s="8" t="e" cm="1">
-        <f t="array" aca="1" ref="B21" ca="1">_xll.QS.CONTEXT.ADD.ZERO.CURVE(Bond_Root,"SOFR",Bond_Pillars,Bond_ZeroRates,"Actual360","Continuous","Annual","Linear",TRUE)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C21" s="5" t="s">
+      <c r="B21" s="10" cm="1" t="str">
+        <f t="array" ref="B21">_xll.QS.CONTEXT.ADD.ZERO.CURVE(Bond_Root,"SOFR",Bond_Pillars,Bond_ZeroRates,"Actual360","Continuous","Annual","Linear",TRUE)</f>
+        <v/>
+      </c>
+      <c r="C21" s="7" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="14" t="str">
-        <f ca="1">SUBSTITUTE(_xlfn.FORMULATEXT(B21),",",", ")</f>
-        <v>=QS.CONTEXT.ADD.ZERO.CURVE(Bond_Root;"SOFR";Bond_Pillars;Bond_ZeroRates;"Actual360";"Continuous";"Annual";"Linear";VERDADERO)</v>
-      </c>
-      <c r="B22" s="14"/>
-      <c r="C22" s="14"/>
+    <row r="22" spans="1:3" ht="33.75" customHeight="1">
+      <c r="A22" s="13" t="str">
+        <f>SUBSTITUTE(_xlfn.FORMULATEXT(B21),",",", ")</f>
+        <v>=QS.CONTEXT.ADD.ZERO.CURVE(Bond_Root, "SOFR", Bond_Pillars, Bond_ZeroRates, "Actual360", "Continuous", "Annual", "Linear", TRUE)</v>
+      </c>
+      <c r="B22" s="13"/>
+      <c r="C22" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -2097,8 +2046,8 @@
     <mergeCell ref="A22:C22"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A4" location="'Start Here'!A1" display="← Start Here" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
-    <hyperlink ref="C4" location="'3 Build'!A1" display="Next → 3 Build" xr:uid="{00000000-0004-0000-0200-000001000000}"/>
+    <hyperlink ref="A4" location="'Start Here'!A1" display="← Start Here"/>
+    <hyperlink ref="C4" location="'3 Build'!A1" display="Next → 3 Build"/>
   </hyperlinks>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape"/>
@@ -2110,311 +2059,311 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <tabColor rgb="FF78909C"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:C46"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="24" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="24" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="34.7109375" style="1" customWidth="1"/>
     <col min="2" max="3" width="48.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+    <row r="1" spans="1:3" ht="38.25" customHeight="1">
+      <c r="A1" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-    </row>
-    <row r="2" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+    </row>
+    <row r="2" spans="1:3" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-    </row>
-    <row r="3" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="16"/>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-    </row>
-    <row r="4" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+    </row>
+    <row r="3" spans="1:3" ht="24" customHeight="1">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+    </row>
+    <row r="4" spans="1:3" ht="36" customHeight="1">
+      <c r="A4" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="6" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+    <row r="6" spans="1:3" ht="36" customHeight="1">
+      <c r="A6" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="5" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:3" ht="38.25" customHeight="1">
+      <c r="A7" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="B7" s="8" t="e" cm="1">
-        <f t="array" aca="1" ref="B7" ca="1">Bond_Root</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C7" s="5" t="s">
+      <c r="B7" s="10">
+        <f>Bond_Root</f>
+        <v/>
+      </c>
+      <c r="C7" s="7" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="str">
-        <f ca="1">SUBSTITUTE(_xlfn.FORMULATEXT(B7),",",", ")</f>
+    <row r="8" spans="1:3" ht="33.75" customHeight="1">
+      <c r="A8" s="13" t="str">
+        <f>SUBSTITUTE(_xlfn.FORMULATEXT(B7),",",", ")</f>
         <v>=Bond_Root</v>
       </c>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-    </row>
-    <row r="10" spans="1:3" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
+    </row>
+    <row r="10" spans="1:3" ht="38.25" customHeight="1">
+      <c r="A10" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="B10" s="8" t="e" cm="1">
-        <f t="array" aca="1" ref="B10" ca="1">_xll.QS.INSTRUMENT.FIXED.RATE.BOND("Bond.Instrument",Bond_Start,Bond_Maturity,"USD",,Bond_Notional,Bond_Coupon,"Actual360","Compounded","Semiannual","Semiannual")</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C10" s="5" t="s">
+      <c r="B10" s="10" cm="1" t="str">
+        <f t="array" ref="B10">_xll.QS.INSTRUMENT.FIXED.RATE.BOND("Bond.Instrument",Bond_Context,Bond_Start,Bond_Maturity,"USD",,Bond_Notional,Bond_Coupon,"Actual360","Compounded","Semiannual","Semiannual")</f>
+        <v/>
+      </c>
+      <c r="C10" s="7" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="str">
-        <f ca="1">SUBSTITUTE(_xlfn.FORMULATEXT(B10),",",", ")</f>
-        <v>=QS.INSTRUMENT.FIXED.RATE.BOND("Bond.Instrument";Bond_Start;Bond_Maturity;"USD";;Bond_Notional;Bond_Coupon;"Actual360";"Compounded";"Semiannual";"Semiannual")</v>
-      </c>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-    </row>
-    <row r="13" spans="1:3" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+    <row r="11" spans="1:3" ht="48" customHeight="1">
+      <c r="A11" s="13" t="str">
+        <f>SUBSTITUTE(_xlfn.FORMULATEXT(B10),",",", ")</f>
+        <v>=QS.INSTRUMENT.FIXED.RATE.BOND("Bond.Instrument", Bond_Context, Bond_Start, Bond_Maturity, "USD", , Bond_Notional, Bond_Coupon, "Actual360", "Compounded", "Semiannual", "Semiannual")</v>
+      </c>
+      <c r="B11" s="13"/>
+      <c r="C11" s="13"/>
+    </row>
+    <row r="13" spans="1:3" ht="38.25" customHeight="1">
+      <c r="A13" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="B13" s="8" t="e" cm="1">
-        <f t="array" aca="1" ref="B13" ca="1">_xll.QS.DISCOUNT.POLICY.FIXED.INCOME("Bond.Policy",Bond_DiscountCurrency,Bond_DiscountIndex)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C13" s="5" t="s">
+      <c r="B13" s="10" cm="1" t="str">
+        <f t="array" ref="B13">_xll.QS.DISCOUNT.POLICY.FIXED.INCOME("Bond.Policy",Bond_DiscountCurrency,Bond_DiscountIndex)</f>
+        <v/>
+      </c>
+      <c r="C13" s="7" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="14" t="str">
-        <f ca="1">SUBSTITUTE(_xlfn.FORMULATEXT(B13),",",", ")</f>
-        <v>=QS.DISCOUNT.POLICY.FIXED.INCOME("Bond.Policy";Bond_DiscountCurrency;Bond_DiscountIndex)</v>
-      </c>
-      <c r="B14" s="14"/>
-      <c r="C14" s="14"/>
-    </row>
-    <row r="16" spans="1:3" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
+    <row r="14" spans="1:3" ht="33.75" customHeight="1">
+      <c r="A14" s="13" t="str">
+        <f>SUBSTITUTE(_xlfn.FORMULATEXT(B13),",",", ")</f>
+        <v>=QS.DISCOUNT.POLICY.FIXED.INCOME("Bond.Policy", Bond_DiscountCurrency, Bond_DiscountIndex)</v>
+      </c>
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
+    </row>
+    <row r="16" spans="1:3" ht="38.25" customHeight="1">
+      <c r="A16" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="B16" s="8" t="e" cm="1">
-        <f t="array" aca="1" ref="B16" ca="1">_xll.QS.PRICER.CREATE("Bond.Pricer","BondPricer",Bond_Policy)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C16" s="5" t="s">
+      <c r="B16" s="10" cm="1" t="str">
+        <f t="array" ref="B16">_xll.QS.PRICER.CREATE("Bond.Pricer","BondPricer",Bond_Policy)</f>
+        <v/>
+      </c>
+      <c r="C16" s="7" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="14" t="str">
-        <f ca="1">SUBSTITUTE(_xlfn.FORMULATEXT(B16),",",", ")</f>
-        <v>=QS.PRICER.CREATE("Bond.Pricer";"BondPricer";Bond_Policy)</v>
-      </c>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
-    </row>
-    <row r="19" spans="1:3" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
+    <row r="17" spans="1:3" ht="33.75" customHeight="1">
+      <c r="A17" s="13" t="str">
+        <f>SUBSTITUTE(_xlfn.FORMULATEXT(B16),",",", ")</f>
+        <v>=QS.PRICER.CREATE("Bond.Pricer", "BondPricer", Bond_Policy)</v>
+      </c>
+      <c r="B17" s="13"/>
+      <c r="C17" s="13"/>
+    </row>
+    <row r="19" spans="1:3" ht="38.25" customHeight="1">
+      <c r="A19" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="B19" s="8" t="e" cm="1">
-        <f t="array" aca="1" ref="B19" ca="1">_xll.QS.TRADE.CREATE("Bond.C01.Trade",Bond_Instrument,Bond_ValuationDate,Bond_Side,,,Bond_C01_Anchor,Bond_C01_AnchorValue)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C19" s="5" t="s">
+      <c r="B19" s="10" cm="1" t="str">
+        <f t="array" ref="B19">_xll.QS.TRADE.CREATE("Bond.C01.Trade",Bond_Context,Bond_Instrument,Bond_ValuationDate,Bond_Side,,,Bond_C01_Anchor,Bond_C01_AnchorValue)</f>
+        <v/>
+      </c>
+      <c r="C19" s="7" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="14" t="str">
-        <f ca="1">SUBSTITUTE(_xlfn.FORMULATEXT(B19),",",", ")</f>
-        <v>=QS.TRADE.CREATE("Bond.C01.Trade";Bond_Instrument;Bond_ValuationDate;Bond_Side;;;Bond_C01_Anchor;Bond_C01_AnchorValue)</v>
-      </c>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14"/>
-    </row>
-    <row r="22" spans="1:3" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
+    <row r="20" spans="1:3" ht="33.75" customHeight="1">
+      <c r="A20" s="13" t="str">
+        <f>SUBSTITUTE(_xlfn.FORMULATEXT(B19),",",", ")</f>
+        <v>=QS.TRADE.CREATE("Bond.C01.Trade", Bond_Context, Bond_Instrument, Bond_ValuationDate, Bond_Side, , , Bond_C01_Anchor, Bond_C01_AnchorValue)</v>
+      </c>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
+    </row>
+    <row r="22" spans="1:3" ht="38.25" customHeight="1">
+      <c r="A22" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="B22" s="8" t="e" cm="1">
-        <f t="array" aca="1" ref="B22" ca="1">_xll.QS.EVALUATE.RESULTS(Bond_Context,Bond_C01_Trade,Bond_Requests,Bond_Pricer)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C22" s="5" t="s">
+      <c r="B22" s="10" cm="1" t="str">
+        <f t="array" ref="B22">_xll.QS.EVALUATE.RESULTS(Bond_Context,Bond_C01_Trade,Bond_Requests,Bond_Pricer)</f>
+        <v/>
+      </c>
+      <c r="C22" s="7" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="14" t="str">
-        <f ca="1">SUBSTITUTE(_xlfn.FORMULATEXT(B22),",",", ")</f>
-        <v>=QS.EVALUATE.RESULTS(Bond_Context;Bond_C01_Trade;Bond_Requests;Bond_Pricer)</v>
-      </c>
-      <c r="B23" s="14"/>
-      <c r="C23" s="14"/>
-    </row>
-    <row r="25" spans="1:3" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="2" t="s">
+    <row r="23" spans="1:3" ht="33.75" customHeight="1">
+      <c r="A23" s="13" t="str">
+        <f>SUBSTITUTE(_xlfn.FORMULATEXT(B22),",",", ")</f>
+        <v>=QS.EVALUATE.RESULTS(Bond_Context, Bond_C01_Trade, Bond_Requests, Bond_Pricer)</v>
+      </c>
+      <c r="B23" s="13"/>
+      <c r="C23" s="13"/>
+    </row>
+    <row r="25" spans="1:3" ht="38.25" customHeight="1">
+      <c r="A25" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="B25" s="8" t="e" cm="1">
-        <f t="array" aca="1" ref="B25" ca="1">_xll.QS.TRADE.CREATE("Bond.C02.Trade",Bond_Instrument,Bond_ValuationDate,Bond_Side,,,Bond_C02_Anchor,Bond_C02_AnchorValue)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C25" s="5" t="s">
+      <c r="B25" s="10" cm="1" t="str">
+        <f t="array" ref="B25">_xll.QS.TRADE.CREATE("Bond.C02.Trade",Bond_Context,Bond_Instrument,Bond_ValuationDate,Bond_Side,,,Bond_C02_Anchor,Bond_C02_AnchorValue)</f>
+        <v/>
+      </c>
+      <c r="C25" s="7" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="14" t="str">
-        <f ca="1">SUBSTITUTE(_xlfn.FORMULATEXT(B25),",",", ")</f>
-        <v>=QS.TRADE.CREATE("Bond.C02.Trade";Bond_Instrument;Bond_ValuationDate;Bond_Side;;;Bond_C02_Anchor;Bond_C02_AnchorValue)</v>
-      </c>
-      <c r="B26" s="14"/>
-      <c r="C26" s="14"/>
-    </row>
-    <row r="28" spans="1:3" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="2" t="s">
+    <row r="26" spans="1:3" ht="33.75" customHeight="1">
+      <c r="A26" s="13" t="str">
+        <f>SUBSTITUTE(_xlfn.FORMULATEXT(B25),",",", ")</f>
+        <v>=QS.TRADE.CREATE("Bond.C02.Trade", Bond_Context, Bond_Instrument, Bond_ValuationDate, Bond_Side, , , Bond_C02_Anchor, Bond_C02_AnchorValue)</v>
+      </c>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+    </row>
+    <row r="28" spans="1:3" ht="38.25" customHeight="1">
+      <c r="A28" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="B28" s="8" t="e" cm="1">
-        <f t="array" aca="1" ref="B28" ca="1">_xll.QS.EVALUATE.RESULTS(Bond_Context,Bond_C02_Trade,Bond_Requests,Bond_Pricer)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C28" s="5" t="s">
+      <c r="B28" s="10" cm="1" t="str">
+        <f t="array" ref="B28">_xll.QS.EVALUATE.RESULTS(Bond_Context,Bond_C02_Trade,Bond_Requests,Bond_Pricer)</f>
+        <v/>
+      </c>
+      <c r="C28" s="7" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="14" t="str">
-        <f ca="1">SUBSTITUTE(_xlfn.FORMULATEXT(B28),",",", ")</f>
-        <v>=QS.EVALUATE.RESULTS(Bond_Context;Bond_C02_Trade;Bond_Requests;Bond_Pricer)</v>
-      </c>
-      <c r="B29" s="14"/>
-      <c r="C29" s="14"/>
-    </row>
-    <row r="31" spans="1:3" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="2" t="s">
+    <row r="29" spans="1:3" ht="33.75" customHeight="1">
+      <c r="A29" s="13" t="str">
+        <f>SUBSTITUTE(_xlfn.FORMULATEXT(B28),",",", ")</f>
+        <v>=QS.EVALUATE.RESULTS(Bond_Context, Bond_C02_Trade, Bond_Requests, Bond_Pricer)</v>
+      </c>
+      <c r="B29" s="13"/>
+      <c r="C29" s="13"/>
+    </row>
+    <row r="31" spans="1:3" ht="38.25" customHeight="1">
+      <c r="A31" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="B31" s="8" t="e" cm="1">
-        <f t="array" aca="1" ref="B31" ca="1">_xll.QS.TRADE.CREATE("Bond.C03.Trade",Bond_Instrument,Bond_ValuationDate,Bond_Side,,,Bond_C03_Anchor,Bond_C03_AnchorValue)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C31" s="5" t="s">
+      <c r="B31" s="10" cm="1" t="str">
+        <f t="array" ref="B31">_xll.QS.TRADE.CREATE("Bond.C03.Trade",Bond_Context,Bond_Instrument,Bond_ValuationDate,Bond_Side,,,Bond_C03_Anchor,Bond_C03_AnchorValue)</f>
+        <v/>
+      </c>
+      <c r="C31" s="7" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="14" t="str">
-        <f ca="1">SUBSTITUTE(_xlfn.FORMULATEXT(B31),",",", ")</f>
-        <v>=QS.TRADE.CREATE("Bond.C03.Trade";Bond_Instrument;Bond_ValuationDate;Bond_Side;;;Bond_C03_Anchor;Bond_C03_AnchorValue)</v>
-      </c>
-      <c r="B32" s="14"/>
-      <c r="C32" s="14"/>
-    </row>
-    <row r="34" spans="1:3" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="2" t="s">
+    <row r="32" spans="1:3" ht="33.75" customHeight="1">
+      <c r="A32" s="13" t="str">
+        <f>SUBSTITUTE(_xlfn.FORMULATEXT(B31),",",", ")</f>
+        <v>=QS.TRADE.CREATE("Bond.C03.Trade", Bond_Context, Bond_Instrument, Bond_ValuationDate, Bond_Side, , , Bond_C03_Anchor, Bond_C03_AnchorValue)</v>
+      </c>
+      <c r="B32" s="13"/>
+      <c r="C32" s="13"/>
+    </row>
+    <row r="34" spans="1:3" ht="38.25" customHeight="1">
+      <c r="A34" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="B34" s="8" t="e" cm="1">
-        <f t="array" aca="1" ref="B34" ca="1">_xll.QS.EVALUATE.RESULTS(Bond_Context,Bond_C03_Trade,Bond_Requests,Bond_Pricer)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C34" s="5" t="s">
+      <c r="B34" s="10" cm="1" t="str">
+        <f t="array" ref="B34">_xll.QS.EVALUATE.RESULTS(Bond_Context,Bond_C03_Trade,Bond_Requests,Bond_Pricer)</f>
+        <v/>
+      </c>
+      <c r="C34" s="7" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="14" t="str">
-        <f ca="1">SUBSTITUTE(_xlfn.FORMULATEXT(B34),",",", ")</f>
-        <v>=QS.EVALUATE.RESULTS(Bond_Context;Bond_C03_Trade;Bond_Requests;Bond_Pricer)</v>
-      </c>
-      <c r="B35" s="14"/>
-      <c r="C35" s="14"/>
-    </row>
-    <row r="39" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="3" t="s">
+    <row r="35" spans="1:3" ht="33.75" customHeight="1">
+      <c r="A35" s="13" t="str">
+        <f>SUBSTITUTE(_xlfn.FORMULATEXT(B34),",",", ")</f>
+        <v>=QS.EVALUATE.RESULTS(Bond_Context, Bond_C03_Trade, Bond_Requests, Bond_Pricer)</v>
+      </c>
+      <c r="B35" s="13"/>
+      <c r="C35" s="13"/>
+    </row>
+    <row r="39" spans="1:3" ht="36" customHeight="1">
+      <c r="A39" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="B39" s="3" t="s">
+      <c r="B39" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="C39" s="3"/>
-    </row>
-    <row r="40" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C39" s="5"/>
+    </row>
+    <row r="40" spans="1:3" ht="24" customHeight="1">
       <c r="A40" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B40" s="8" t="e">
-        <f ca="1">Bond_C01_Result</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B40" s="10">
+        <f>Bond_C01_Result</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="24" customHeight="1">
       <c r="A41" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B41" s="8" t="e">
-        <f ca="1">Bond_C02_Result</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B41" s="10">
+        <f>Bond_C02_Result</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="24" customHeight="1">
       <c r="A42" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B42" s="8" t="e">
-        <f ca="1">Bond_C03_Result</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="2" t="s">
+      <c r="B42" s="10">
+        <f>Bond_C03_Result</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45" spans="1:3" ht="38.25" customHeight="1">
+      <c r="A45" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="B45" s="8" t="e">
-        <f ca="1">INDEX(Bond_ResultHandles,MATCH(Bond_SelectedCase,Bond_CaseNames,0))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C45" s="5" t="s">
+      <c r="B45" s="10">
+        <f>INDEX(Bond_ResultHandles,MATCH(Bond_SelectedCase,Bond_CaseNames,0))</f>
+        <v/>
+      </c>
+      <c r="C45" s="7" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="14" t="str">
-        <f ca="1">SUBSTITUTE(_xlfn.FORMULATEXT(B45),",",", ")</f>
-        <v>=INDICE(Bond_ResultHandles;COINCIDIR(Bond_SelectedCase;Bond_CaseNames;0))</v>
-      </c>
-      <c r="B46" s="14"/>
-      <c r="C46" s="14"/>
+    <row r="46" spans="1:3" ht="33.75" customHeight="1">
+      <c r="A46" s="13" t="str">
+        <f>SUBSTITUTE(_xlfn.FORMULATEXT(B45),",",", ")</f>
+        <v>=INDEX(Bond_ResultHandles, MATCH(Bond_SelectedCase, Bond_CaseNames, 0))</v>
+      </c>
+      <c r="B46" s="13"/>
+      <c r="C46" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -2423,18 +2372,18 @@
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="A14:C14"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="A46:C46"/>
     <mergeCell ref="A17:C17"/>
     <mergeCell ref="A20:C20"/>
     <mergeCell ref="A23:C23"/>
     <mergeCell ref="A26:C26"/>
     <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="A46:C46"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A4" location="'Start Here'!A1" display="← Start Here" xr:uid="{00000000-0004-0000-0300-000000000000}"/>
-    <hyperlink ref="C4" location="'4 Results'!A1" display="Next → 4 Results" xr:uid="{00000000-0004-0000-0300-000001000000}"/>
+    <hyperlink ref="A4" location="'Start Here'!A1" display="← Start Here"/>
+    <hyperlink ref="C4" location="'4 Results'!A1" display="Next → 4 Results"/>
   </hyperlinks>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape"/>
@@ -2446,13 +2395,13 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <tabColor rgb="FF21845B"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="24" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="24" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="30.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="22.7109375" style="1" customWidth="1"/>
@@ -2460,176 +2409,176 @@
     <col min="5" max="6" width="16.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+    <row r="1" spans="1:6" ht="38.25" customHeight="1">
+      <c r="A1" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-    </row>
-    <row r="2" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+    </row>
+    <row r="2" spans="1:6" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-    </row>
-    <row r="3" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="16"/>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-    </row>
-    <row r="4" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+    </row>
+    <row r="3" spans="1:6" ht="24" customHeight="1">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+    </row>
+    <row r="4" spans="1:6" ht="36" customHeight="1">
+      <c r="A4" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="6" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+    <row r="6" spans="1:6" ht="36" customHeight="1">
+      <c r="A6" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="5" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="33.75" customHeight="1">
       <c r="A7" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B7" s="11" t="e" cm="1">
-        <f t="array" aca="1" ref="B7" ca="1">_xll.QS.RESULT.VALUE(Bond_C01_Result)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C7" s="12" t="e" cm="1">
-        <f t="array" aca="1" ref="C7" ca="1">_xll.QS.RESULT.MODIFIED.DURATION(Bond_C01_Result)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D7" s="13" t="e" cm="1">
-        <f t="array" aca="1" ref="D7" ca="1">_xll.QS.RESULT.Z.SPREAD(Bond_C01_Result)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E7" s="4" t="s">
+      <c r="B7" s="14" cm="1" t="str">
+        <f t="array" ref="B7">_xll.QS.RESULT.VALUE(Bond_C01_Result)</f>
+        <v/>
+      </c>
+      <c r="C7" s="15" cm="1" t="str">
+        <f t="array" ref="C7">_xll.QS.RESULT.MODIFIED.DURATION(Bond_C01_Result)</f>
+        <v/>
+      </c>
+      <c r="D7" s="16" cm="1" t="str">
+        <f t="array" ref="D7">_xll.QS.RESULT.Z.SPREAD(Bond_C01_Result)</f>
+        <v/>
+      </c>
+      <c r="E7" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="6" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="33.75" customHeight="1">
       <c r="A8" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B8" s="11" t="e" cm="1">
-        <f t="array" aca="1" ref="B8" ca="1">_xll.QS.RESULT.VALUE(Bond_C02_Result)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C8" s="12" t="e" cm="1">
-        <f t="array" aca="1" ref="C8" ca="1">_xll.QS.RESULT.MODIFIED.DURATION(Bond_C02_Result)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D8" s="13" t="e" cm="1">
-        <f t="array" aca="1" ref="D8" ca="1">_xll.QS.RESULT.Z.SPREAD(Bond_C02_Result)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E8" s="4" t="s">
+      <c r="B8" s="14" cm="1" t="str">
+        <f t="array" ref="B8">_xll.QS.RESULT.VALUE(Bond_C02_Result)</f>
+        <v/>
+      </c>
+      <c r="C8" s="15" cm="1" t="str">
+        <f t="array" ref="C8">_xll.QS.RESULT.MODIFIED.DURATION(Bond_C02_Result)</f>
+        <v/>
+      </c>
+      <c r="D8" s="16" cm="1" t="str">
+        <f t="array" ref="D8">_xll.QS.RESULT.Z.SPREAD(Bond_C02_Result)</f>
+        <v/>
+      </c>
+      <c r="E8" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="6" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" ht="33.75" customHeight="1">
       <c r="A9" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B9" s="11" t="e" cm="1">
-        <f t="array" aca="1" ref="B9" ca="1">_xll.QS.RESULT.VALUE(Bond_C03_Result)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C9" s="12" t="e" cm="1">
-        <f t="array" aca="1" ref="C9" ca="1">_xll.QS.RESULT.MODIFIED.DURATION(Bond_C03_Result)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D9" s="13" t="e" cm="1">
-        <f t="array" aca="1" ref="D9" ca="1">_xll.QS.RESULT.Z.SPREAD(Bond_C03_Result)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E9" s="4" t="s">
+      <c r="B9" s="14" cm="1" t="str">
+        <f t="array" ref="B9">_xll.QS.RESULT.VALUE(Bond_C03_Result)</f>
+        <v/>
+      </c>
+      <c r="C9" s="15" cm="1" t="str">
+        <f t="array" ref="C9">_xll.QS.RESULT.MODIFIED.DURATION(Bond_C03_Result)</f>
+        <v/>
+      </c>
+      <c r="D9" s="16" cm="1" t="str">
+        <f t="array" ref="D9">_xll.QS.RESULT.Z.SPREAD(Bond_C03_Result)</f>
+        <v/>
+      </c>
+      <c r="E9" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F9" s="6" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+    <row r="13" spans="1:6" ht="24" customHeight="1">
+      <c r="A13" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="C13" s="19" t="s">
+      <c r="C13" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
-    </row>
-    <row r="14" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
-    </row>
-    <row r="17" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="19" t="s">
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+    </row>
+    <row r="14" spans="1:6" ht="24" customHeight="1">
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+    </row>
+    <row r="17" spans="1:6" ht="24" customHeight="1">
+      <c r="A17" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="B17" s="19"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="19"/>
-    </row>
-    <row r="18" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="19"/>
-      <c r="B18" s="19"/>
-      <c r="C18" s="19"/>
-      <c r="D18" s="19"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="19"/>
-    </row>
-    <row r="19" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="19"/>
-      <c r="B19" s="19"/>
-      <c r="C19" s="19"/>
-      <c r="D19" s="19"/>
-      <c r="E19" s="19"/>
-      <c r="F19" s="19"/>
+      <c r="B17" s="7"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+    </row>
+    <row r="18" spans="1:6" ht="24" customHeight="1">
+      <c r="A18" s="7"/>
+      <c r="B18" s="7"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+    </row>
+    <row r="19" spans="1:6" ht="24" customHeight="1">
+      <c r="A19" s="7"/>
+      <c r="B19" s="7"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2639,19 +2588,19 @@
     <mergeCell ref="A17:F19"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B13" xr:uid="{00000000-0002-0000-0400-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B13">
       <formula1>Bond_CaseNames</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="A4" location="'Start Here'!A1" display="← Start Here" xr:uid="{00000000-0004-0000-0400-000000000000}"/>
-    <hyperlink ref="F4" location="'5 Cashflows'!A1" display="Next → 5 Cashflows" xr:uid="{00000000-0004-0000-0400-000001000000}"/>
-    <hyperlink ref="E7" location="'1 Inputs'!C17" display="Edit →" xr:uid="{00000000-0004-0000-0400-000002000000}"/>
-    <hyperlink ref="F7" location="'3 Build'!A19" display="Build →" xr:uid="{00000000-0004-0000-0400-000003000000}"/>
-    <hyperlink ref="E8" location="'1 Inputs'!C18" display="Edit →" xr:uid="{00000000-0004-0000-0400-000004000000}"/>
-    <hyperlink ref="F8" location="'3 Build'!A25" display="Build →" xr:uid="{00000000-0004-0000-0400-000005000000}"/>
-    <hyperlink ref="E9" location="'1 Inputs'!C19" display="Edit →" xr:uid="{00000000-0004-0000-0400-000006000000}"/>
-    <hyperlink ref="F9" location="'3 Build'!A31" display="Build →" xr:uid="{00000000-0004-0000-0400-000007000000}"/>
+    <hyperlink ref="A4" location="'Start Here'!A1" display="← Start Here"/>
+    <hyperlink ref="F4" location="'5 Cashflows'!A1" display="Next → 5 Cashflows"/>
+    <hyperlink ref="E7" location="'1 Inputs'!C17" display="Edit →"/>
+    <hyperlink ref="F7" location="'3 Build'!A19" display="Build →"/>
+    <hyperlink ref="E8" location="'1 Inputs'!C18" display="Edit →"/>
+    <hyperlink ref="F8" location="'3 Build'!A25" display="Build →"/>
+    <hyperlink ref="E9" location="'1 Inputs'!C19" display="Edit →"/>
+    <hyperlink ref="F9" location="'3 Build'!A31" display="Build →"/>
   </hyperlinks>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape"/>
@@ -2662,85 +2611,85 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <tabColor rgb="FF78909C"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="24" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="24" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="28.7109375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="11" customWidth="1"/>
-    <col min="4" max="4" width="12.7109375" style="13" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" style="12" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" style="14" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" style="16" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" style="15" customWidth="1"/>
     <col min="6" max="6" width="12.7109375" style="1" customWidth="1"/>
-    <col min="7" max="8" width="12.7109375" style="13" customWidth="1"/>
+    <col min="7" max="8" width="12.7109375" style="16" customWidth="1"/>
     <col min="9" max="9" width="8.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+    <row r="1" spans="1:9" ht="38.25" customHeight="1">
+      <c r="A1" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
-    </row>
-    <row r="2" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+    </row>
+    <row r="2" spans="1:9" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16"/>
-      <c r="I2" s="16"/>
-    </row>
-    <row r="3" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="16"/>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
-      <c r="I3" s="16"/>
-    </row>
-    <row r="4" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+    </row>
+    <row r="3" spans="1:9" ht="24" customHeight="1">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+    </row>
+    <row r="4" spans="1:9" ht="36" customHeight="1">
+      <c r="A4" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="I4" s="4" t="s">
+      <c r="I4" s="6" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="24" customHeight="1">
       <c r="A6" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="B6" s="7" t="str">
+      <c r="B6" s="9">
         <f>Bond_SelectedCase</f>
-        <v>Zero spread</v>
-      </c>
-      <c r="C6" s="4" t="s">
+        <v/>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="e" cm="1">
-        <f t="array" aca="1" ref="A7" ca="1">_xll.QS.RESULT.CASHFLOWS(Bond_SelectedResult)</f>
-        <v>#VALUE!</v>
+    <row r="7" spans="1:9" ht="24" customHeight="1">
+      <c r="A7" s="1" cm="1" t="str">
+        <f t="array" ref="A7">_xll.QS.RESULT.CASHFLOWS(Bond_SelectedResult)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -2749,9 +2698,9 @@
     <mergeCell ref="A2:I3"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A4" location="'Start Here'!A1" display="← Start Here" xr:uid="{00000000-0004-0000-0500-000000000000}"/>
-    <hyperlink ref="I4" location="'6 Risk'!A1" display="Next → 6 Risk" xr:uid="{00000000-0004-0000-0500-000001000000}"/>
-    <hyperlink ref="C6" location="'4 Results'!B13" display="Change case →" xr:uid="{00000000-0004-0000-0500-000002000000}"/>
+    <hyperlink ref="A4" location="'Start Here'!A1" display="← Start Here"/>
+    <hyperlink ref="I4" location="'6 Risk'!A1" display="Next → 6 Risk"/>
+    <hyperlink ref="C6" location="'4 Results'!B13" display="Change case →"/>
   </hyperlinks>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape"/>
@@ -2762,59 +2711,59 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <tabColor rgb="FF78909C"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="24" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="24" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="62.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="24.7109375" style="11" customWidth="1"/>
+    <col min="2" max="2" width="24.7109375" style="14" customWidth="1"/>
     <col min="3" max="3" width="24.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+    <row r="1" spans="1:3" ht="38.25" customHeight="1">
+      <c r="A1" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-    </row>
-    <row r="2" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+    </row>
+    <row r="2" spans="1:3" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-    </row>
-    <row r="3" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="16"/>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-    </row>
-    <row r="4" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+    </row>
+    <row r="3" spans="1:3" ht="24" customHeight="1">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+    </row>
+    <row r="4" spans="1:3" ht="24" customHeight="1">
+      <c r="A4" s="6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="24" customHeight="1">
       <c r="A6" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="B6" s="7" t="str">
+      <c r="B6" s="9">
         <f>Bond_SelectedCase</f>
-        <v>Zero spread</v>
-      </c>
-      <c r="C6" s="4" t="s">
+        <v/>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="e" cm="1">
-        <f t="array" aca="1" ref="A7" ca="1">_xll.QS.RESULT.SENSITIVITIES(Bond_SelectedResult)</f>
-        <v>#VALUE!</v>
+    <row r="7" spans="1:3" ht="24" customHeight="1">
+      <c r="A7" s="1" cm="1" t="str">
+        <f t="array" ref="A7">_xll.QS.RESULT.SENSITIVITIES(Bond_SelectedResult)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -2823,8 +2772,8 @@
     <mergeCell ref="A2:C3"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A4" location="'Start Here'!A1" display="← Start Here" xr:uid="{00000000-0004-0000-0600-000000000000}"/>
-    <hyperlink ref="C6" location="'4 Results'!B13" display="Change case →" xr:uid="{00000000-0004-0000-0600-000001000000}"/>
+    <hyperlink ref="A4" location="'Start Here'!A1" display="← Start Here"/>
+    <hyperlink ref="C6" location="'4 Results'!B13" display="Change case →"/>
   </hyperlinks>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape"/>

</xml_diff>